<commit_message>
Corregir formato del excel de calificaciones (celdas numericas y encabezados)
</commit_message>
<xml_diff>
--- a/Moviles 1/Calificaciones_Tareas.xlsx
+++ b/Moviles 1/Calificaciones_Tareas.xlsx
@@ -102,543 +102,578 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CALIFICACIONES DE TAREAS - Moviles 1 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CALIFICACIONES DE TAREAS - Moviles 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escala 0.0 a 5.0  |  El mejor proyecto de cada tarea = 5.0  |  No incluye Parcial 1 (ya calificado por el docente) 0</t>
+          <t xml:space="preserve">Escala 0.0 a 5.0  |  El mejor proyecto de cada tarea = 5.0  |  No incluye Parcial 1 (ya calificado por el docente)</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taller Lista Tareas (Kotlin)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lista Tareas (Flutter)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pokemon / Pokedex</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App Notas</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App Clima</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ejercicios Kotlin</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Promedio Tareas</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luis Miguel Franco Perez 0</t>
+          <t xml:space="preserve">Luis Miguel Franco Perez</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>4.2 3</v>
-      </c>
-      <c r="D5">
-        <v>4.8 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="C5" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="D5" s="3">
+        <v>4.8</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H5">
-        <v>4.5 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H5" s="3">
+        <v>4.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sofia Calvijo Zuluaga 0</t>
+          <t xml:space="preserve">Sofia Calvijo Zuluaga</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin entregas 0</t>
+          <t xml:space="preserve">Sin entregas</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sergio Andres Rodriguez Triana 0</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>4.9 3</v>
+          <t xml:space="preserve">Sergio Andres Rodriguez Triana</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <v>4.9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="D7">
-        <v>4.7 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D7" s="3">
+        <v>4.7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H7">
-        <v>4.8 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H7" s="3">
+        <v>4.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Joiner Pineda Torres 0</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>4.5 3</v>
+          <t xml:space="preserve">Joiner Pineda Torres</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <v>4.5</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H8">
-        <v>4.5 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H8" s="3">
+        <v>4.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jeison David Gomez Hernandez 0</t>
+          <t xml:space="preserve">Jeison David Gomez Hernandez</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin entregas 0</t>
+          <t xml:space="preserve">Sin entregas</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Julian David Rodriguez Llano 0</t>
+          <t xml:space="preserve">Julian David Rodriguez Llano</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>4.6 3</v>
-      </c>
-      <c r="D10">
-        <v>4 3</v>
-      </c>
-      <c r="E10">
-        <v>4 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="C10" s="3">
+        <v>4.6</v>
+      </c>
+      <c r="D10" s="3">
+        <v>4</v>
+      </c>
+      <c r="E10" s="3">
+        <v>4</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H10">
-        <v>4.2 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H10" s="3">
+        <v>4.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Veronica Clavijo Zuluaga 0</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>4.3 3</v>
+          <t xml:space="preserve">Veronica Clavijo Zuluaga</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <v>4.3</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H11">
-        <v>4.3 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H11" s="3">
+        <v>4.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gustavo Adolfo Marin Munoz 0</t>
+          <t xml:space="preserve">Gustavo Adolfo Marin Munoz</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>4.8 3</v>
-      </c>
-      <c r="D12">
-        <v>5 3</v>
-      </c>
-      <c r="E12">
-        <v>5 3</v>
-      </c>
-      <c r="F12">
-        <v>5 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="C12" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="D12" s="3">
+        <v>5</v>
+      </c>
+      <c r="E12" s="3">
+        <v>5</v>
+      </c>
+      <c r="F12" s="3">
+        <v>5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H12">
-        <v>4.95 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H12" s="3">
+        <v>4.95</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vanessa Miranda 0</t>
+          <t xml:space="preserve">Vanessa Miranda</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin entregas 0</t>
+          <t xml:space="preserve">Sin entregas</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Juan Camilo Ganan Blandon 0</t>
-        </is>
-      </c>
-      <c r="B14">
-        <v>4 3</v>
+          <t xml:space="preserve">Juan Camilo Ganan Blandon</t>
+        </is>
+      </c>
+      <c r="B14" s="3">
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="D14">
-        <v>4.6 3</v>
-      </c>
-      <c r="E14">
-        <v>4 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D14" s="3">
+        <v>4.6</v>
+      </c>
+      <c r="E14" s="3">
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="G14">
-        <v>5 3</v>
-      </c>
-      <c r="H14">
-        <v>4.4 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G14" s="3">
+        <v>5</v>
+      </c>
+      <c r="H14" s="3">
+        <v>4.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Juan Mateo Garcia Martinez 0</t>
-        </is>
-      </c>
-      <c r="B15">
-        <v>4.7 3</v>
+          <t xml:space="preserve">Juan Mateo Garcia Martinez</t>
+        </is>
+      </c>
+      <c r="B15" s="3">
+        <v>4.7</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="G15">
-        <v>5 3</v>
-      </c>
-      <c r="H15">
-        <v>4.85 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G15" s="3">
+        <v>5</v>
+      </c>
+      <c r="H15" s="3">
+        <v>4.85</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luis Miguel Castillo Castano 0</t>
-        </is>
-      </c>
-      <c r="B16">
-        <v>1 3</v>
+          <t xml:space="preserve">Luis Miguel Castillo Castano</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H16">
-        <v>1 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H16" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Angelo Franco Orozco 0</t>
-        </is>
-      </c>
-      <c r="B17">
-        <v>5 3</v>
+          <t xml:space="preserve">Angelo Franco Orozco</t>
+        </is>
+      </c>
+      <c r="B17" s="3">
+        <v>5</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H17">
-        <v>5 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H17" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bryan Steven Salinas Mahecha 0</t>
+          <t xml:space="preserve">Bryan Steven Salinas Mahecha</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="C18">
-        <v>5 3</v>
-      </c>
-      <c r="D18">
-        <v>4.3 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="C18" s="3">
+        <v>5</v>
+      </c>
+      <c r="D18" s="3">
+        <v>4.3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="F18">
-        <v>4.5 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F18" s="3">
+        <v>4.5</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 0</t>
-        </is>
-      </c>
-      <c r="H18">
-        <v>4.6 3</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H18" s="3">
+        <v>4.6</v>
       </c>
     </row>
   </sheetData>
@@ -655,24 +690,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAREA 1 - Taller Lista de Tareas (Android Studio / Kotlin) 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAREA 1 - Taller Lista de Tareas (Android Studio / Kotlin)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rubrica: completar TODO del TareaAdapter (RecyclerView/ViewBinding) y MainActivity (agregar/eliminar/contador). Mejor proyecto = 5.0 0</t>
+          <t xml:space="preserve">Rubrica: completar TODO del TareaAdapter (RecyclerView/ViewBinding) y MainActivity (agregar/eliminar/contador). Mejor proyecto = 5.0</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle / Justificacion</t>
         </is>
       </c>
     </row>
@@ -687,12 +737,12 @@
           <t xml:space="preserve">Windfull13/Programacion-moviles-2</t>
         </is>
       </c>
-      <c r="C5">
-        <v>5 3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Todos los TODO del Adapter y MainActivity completos. Extras: persistencia con SharedPreferences+Gson, onSaveInstanceState/restaurarEstado, strings en res/values (i18n), setOnCheckedChangeListener(null) anti-reciclaje. El mejor acabado. 4</t>
+      <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Todos los TODO del Adapter y MainActivity completos. Extras: persistencia con SharedPreferences+Gson, onSaveInstanceState/restaurarEstado, strings en res/values (i18n), setOnCheckedChangeListener(null) anti-reciclaje. El mejor acabado.</t>
         </is>
       </c>
     </row>
@@ -707,12 +757,12 @@
           <t xml:space="preserve">SERGIO-TRIANA/CodigoClaseDispositivosMoviles (Tarea_6)</t>
         </is>
       </c>
-      <c r="C6">
-        <v>4.9 3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adapter 4/4 y MainActivity 13/13. Extra: lambda onToggle (contador refresca al marcar) y archivo Respuestas.kt con las 5 preguntas de cierre. Sin persistencia. 4</t>
+      <c r="C6" s="3">
+        <v>4.9</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adapter 4/4 y MainActivity 13/13. Extra: lambda onToggle (contador refresca al marcar) y archivo Respuestas.kt con las 5 preguntas de cierre. Sin persistencia.</t>
         </is>
       </c>
     </row>
@@ -727,12 +777,12 @@
           <t xml:space="preserve">Jumgarciama/ListaDeTareas</t>
         </is>
       </c>
-      <c r="C7">
-        <v>4.7 3</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adapter 4/4 y MainActivity 13/13. Buen detalle: limpia el listener con setOnCheckedChangeListener(null) para evitar bug de reciclaje. Sin onToggle ni contador inicial. 4</t>
+      <c r="C7" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adapter 4/4 y MainActivity 13/13. Buen detalle: limpia el listener con setOnCheckedChangeListener(null) para evitar bug de reciclaje. Sin onToggle ni contador inicial.</t>
         </is>
       </c>
     </row>
@@ -747,12 +797,12 @@
           <t xml:space="preserve">JoinerPineda/Taller-Android-Kotlin</t>
         </is>
       </c>
-      <c r="C8">
-        <v>4.5 3</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TODO completos y funcionales. README excelente con preguntas respondidas. Detalles: sin lambda onToggle y no llama actualizarContador() en onCreate (contador no refresca al marcar). 4</t>
+      <c r="C8" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TODO completos y funcionales. README excelente con preguntas respondidas. Detalles: sin lambda onToggle y no llama actualizarContador() en onCreate (contador no refresca al marcar).</t>
         </is>
       </c>
     </row>
@@ -767,12 +817,12 @@
           <t xml:space="preserve">Veritosclavijo/taller-lista-tareas</t>
         </is>
       </c>
-      <c r="C9">
-        <v>4.3 3</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Los 13 TODO completos, version base limpia y funcional. Sin extras. Archivos Tarea.kt/TareaAdapter.kt mal ubicados en java/ raiz (funciona igual). 4</t>
+      <c r="C9" s="3">
+        <v>4.3</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los 13 TODO completos, version base limpia y funcional. Sin extras. Archivos Tarea.kt/TareaAdapter.kt mal ubicados en java/ raiz (funciona igual).</t>
         </is>
       </c>
     </row>
@@ -787,12 +837,12 @@
           <t xml:space="preserve">JuanCamiloGanan/Programacion-para-dispositivos-moviles (Lista de Tareas)</t>
         </is>
       </c>
-      <c r="C10">
-        <v>4 3</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TODO completos y funcional, pero el codigo es identico al de Veronica Clavijo (mismos archivos y estructura). Penalizacion por evidencia de codigo compartido/copiado. 4</t>
+      <c r="C10" s="3">
+        <v>4</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TODO completos y funcional, pero el codigo es identico al de Veronica Clavijo (mismos archivos y estructura). Penalizacion por evidencia de codigo compartido/copiado.</t>
         </is>
       </c>
     </row>
@@ -807,12 +857,12 @@
           <t xml:space="preserve">lmcastilloc04/Taller_android_studio_kotlin</t>
         </is>
       </c>
-      <c r="C11">
-        <v>1 3</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Entrega vacia: 0/4 TODO del Adapter y 0/13 de MainActivity (solo el esqueleto con comentarios). No compila como app funcional. Subio ademas la guia del profesor como entregable. 4</t>
+      <c r="C11" s="3">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrega vacia: 0/4 TODO del Adapter y 0/13 de MainActivity (solo el esqueleto con comentarios). No compila como app funcional. Subio ademas la guia del profesor como entregable.</t>
         </is>
       </c>
     </row>
@@ -830,24 +880,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAREA 2 - App Lista de Tareas (Flutter) 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAREA 2 - App Lista de Tareas (Flutter)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rubrica: CRUD de tareas (agregar/eliminar/toggle), contador, validacion, manejo de estado, separacion de codigo. Mejor proyecto = 5.0 0</t>
+          <t xml:space="preserve">Rubrica: CRUD de tareas (agregar/eliminar/toggle), contador, validacion, manejo de estado, separacion de codigo. Mejor proyecto = 5.0</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle / Justificacion</t>
         </is>
       </c>
     </row>
@@ -862,12 +927,12 @@
           <t xml:space="preserve">BSM2003/Dispositivos_Moviles (lista_tarea)</t>
         </is>
       </c>
-      <c r="C5">
-        <v>5 3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CRUD completo (agregar/eliminar/editar inline/toggle), contador de pendientes, categorias con dropdown y color, persistencia con shared_preferences (toJson/fromJson), uuid. Separacion en models/screens/widgets. El mas completo. 4</t>
+      <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRUD completo (agregar/eliminar/editar inline/toggle), contador de pendientes, categorias con dropdown y color, persistencia con shared_preferences (toJson/fromJson), uuid. Separacion en models/screens/widgets. El mas completo.</t>
         </is>
       </c>
     </row>
@@ -882,12 +947,12 @@
           <t xml:space="preserve">Marin708/Talleres_Dispositivos_moviles (TRABAJO_4)</t>
         </is>
       </c>
-      <c r="C6">
-        <v>4.8 3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CRUD completo con filtros (todas/pendientes/completadas), etiquetas (enum con colores), contador y tachado. Estado en memoria. Muy buen nivel. 4</t>
+      <c r="C6" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRUD completo con filtros (todas/pendientes/completadas), etiquetas (enum con colores), contador y tachado. Estado en memoria. Muy buen nivel.</t>
         </is>
       </c>
     </row>
@@ -902,12 +967,12 @@
           <t xml:space="preserve">DavidLlano2004/flutter (taller_flutter)</t>
         </is>
       </c>
-      <c r="C7">
-        <v>4.6 3</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CRUD funcional: agregar, eliminar, toggle, contador, tachado, validacion con SnackBar. Bien separado en models/screens/widgets (Tarea con copyWith/==/hashCode). Estado en memoria. 4</t>
+      <c r="C7" s="3">
+        <v>4.6</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRUD funcional: agregar, eliminar, toggle, contador, tachado, validacion con SnackBar. Bien separado en models/screens/widgets (Tarea con copyWith/==/hashCode). Estado en memoria.</t>
         </is>
       </c>
     </row>
@@ -922,12 +987,12 @@
           <t xml:space="preserve">LuisMiguelFP/Crud_Tareas_flutter</t>
         </is>
       </c>
-      <c r="C8">
-        <v>4.2 3</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CRUD completo + editar (AlertDialog), contador total/completadas, estado vacio amigable. Funcional y bien comentado pero todo en un solo main.dart (sin separacion) y sin persistencia. 4</t>
+      <c r="C8" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRUD completo + editar (AlertDialog), contador total/completadas, estado vacio amigable. Funcional y bien comentado pero todo en un solo main.dart (sin separacion) y sin persistencia.</t>
         </is>
       </c>
     </row>
@@ -945,24 +1010,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAREA 3 - Ejercicio Pokemon / Pokedex (Flutter) 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAREA 3 - Ejercicio Pokemon / Pokedex (Flutter)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rubrica: consumo de PokeAPI, modelos fromJson, busqueda, manejo de estados/errores, UI y arquitectura. Mejor proyecto = 5.0 0</t>
+          <t xml:space="preserve">Rubrica: consumo de PokeAPI, modelos fromJson, busqueda, manejo de estados/errores, UI y arquitectura. Mejor proyecto = 5.0</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle / Justificacion</t>
         </is>
       </c>
     </row>
@@ -977,12 +1057,12 @@
           <t xml:space="preserve">Marin708/Talleres_Dispositivos_moviles (TRABAJO_2)</t>
         </is>
       </c>
-      <c r="C5">
-        <v>5 3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pokedex completa: PokeApiService, modelos, cadena evolutiva, busqueda, recientes con SharedPreferences, google_fonts y UI muy pulida (CustomPainter). Feature-rich. El mejor. 4</t>
+      <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pokedex completa: PokeApiService, modelos, cadena evolutiva, busqueda, recientes con SharedPreferences, google_fonts y UI muy pulida (CustomPainter). Feature-rich. El mejor.</t>
         </is>
       </c>
     </row>
@@ -997,12 +1077,12 @@
           <t xml:space="preserve">LuisMiguelFP/pokedex_flutter</t>
         </is>
       </c>
-      <c r="C6">
-        <v>4.8 3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Consume PokeAPI real, modelo Pokemon.fromJson + Stat, busqueda por nombre/numero con chips, manejo de 404/errores, UI con fondo por tipo y stats. Arquitectura models/services/screens/widgets/utils. README propio. 4</t>
+      <c r="C6" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consume PokeAPI real, modelo Pokemon.fromJson + Stat, busqueda por nombre/numero con chips, manejo de 404/errores, UI con fondo por tipo y stats. Arquitectura models/services/screens/widgets/utils. README propio.</t>
         </is>
       </c>
     </row>
@@ -1017,12 +1097,12 @@
           <t xml:space="preserve">SERGIO-TRIANA/CodigoClaseDispositivosMoviles (PokemonConsulta)</t>
         </is>
       </c>
-      <c r="C7">
-        <v>4.7 3</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pokedex Flutter real (PokeAPI), capas limpias (models/services/screens/widgets/utils), busqueda por nombre o numero, maneja 404, Material3. 4</t>
+      <c r="C7" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pokedex Flutter real (PokeAPI), capas limpias (models/services/screens/widgets/utils), busqueda por nombre o numero, maneja 404, Material3.</t>
         </is>
       </c>
     </row>
@@ -1037,12 +1117,12 @@
           <t xml:space="preserve">JuanCamiloGanan/Programacion-para-dispositivos-moviles (Ejercicio pokemos)</t>
         </is>
       </c>
-      <c r="C8">
-        <v>4.6 3</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App Pokemon con arquitectura limpia (data/repositories, domain/usecases, dto, presentation), usa Dio, pokemon aleatorio + busqueda. El mas ingenieril. 4</t>
+      <c r="C8" s="3">
+        <v>4.6</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App Pokemon con arquitectura limpia (data/repositories, domain/usecases, dto, presentation), usa Dio, pokemon aleatorio + busqueda. El mas ingenieril.</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1137,12 @@
           <t xml:space="preserve">BSM2003/Dispositivos_Moviles (Pokemon_Search)</t>
         </is>
       </c>
-      <c r="C9">
-        <v>4.3 3</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PokeAPI via Dio, modelo Pokemon muy completo (sprites/types/stats), busqueda con FutureBuilder, ExpandableFab. Mezcla el ejercicio con un contador demo en la pantalla principal. 4</t>
+      <c r="C9" s="3">
+        <v>4.3</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PokeAPI via Dio, modelo Pokemon muy completo (sprites/types/stats), busqueda con FutureBuilder, ExpandableFab. Mezcla el ejercicio con un contador demo en la pantalla principal.</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1157,12 @@
           <t xml:space="preserve">DavidLlano2004/flutter (Poke_Api)</t>
         </is>
       </c>
-      <c r="C10">
-        <v>4 3</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App Pokemon funcional (PokeAPI, pokemon aleatorio 1-1025), colores por tipo, UI tematica. Todo en un main.dart (sin separacion) y sin README. 4</t>
+      <c r="C10" s="3">
+        <v>4</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App Pokemon funcional (PokeAPI, pokemon aleatorio 1-1025), colores por tipo, UI tematica. Todo en un main.dart (sin separacion) y sin README.</t>
         </is>
       </c>
     </row>
@@ -1100,24 +1180,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAREA 4 - App de Notas (Flutter) 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAREA 4 - App de Notas (Flutter)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rubrica: consumo de API (jsonplaceholder), listar notas, crear nota, UI. Mejor proyecto = 5.0 0</t>
+          <t xml:space="preserve">Rubrica: consumo de API (jsonplaceholder), listar notas, crear nota, UI. Mejor proyecto = 5.0</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle / Justificacion</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1227,12 @@
           <t xml:space="preserve">Marin708/Talleres_Dispositivos_moviles (TRABAJO_3)</t>
         </is>
       </c>
-      <c r="C5">
-        <v>5 3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App de notas desde jsonplaceholder (GET 10 posts), agregar nota local (create en memoria), buscar por ID, UI cuidada con paleta propia. El mejor. 4</t>
+      <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App de notas desde jsonplaceholder (GET 10 posts), agregar nota local (create en memoria), buscar por ID, UI cuidada con paleta propia. El mejor.</t>
         </is>
       </c>
     </row>
@@ -1152,12 +1247,12 @@
           <t xml:space="preserve">DavidLlano2004/flutter (Notes_app)</t>
         </is>
       </c>
-      <c r="C6">
-        <v>4 3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App de notas Flutter (jsonplaceholder GET + create local + dialog), funcional. El main.dart es identico al de Juan Camilo Ganan: evidencia de codigo compartido (penalizacion). 4</t>
+      <c r="C6" s="3">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App de notas Flutter (jsonplaceholder GET + create local + dialog), funcional. El main.dart es identico al de Juan Camilo Ganan: evidencia de codigo compartido (penalizacion).</t>
         </is>
       </c>
     </row>
@@ -1172,12 +1267,12 @@
           <t xml:space="preserve">JuanCamiloGanan/Programacion-para-dispositivos-moviles (Ejercicio notas)</t>
         </is>
       </c>
-      <c r="C7">
-        <v>4 3</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App de notas Flutter (jsonplaceholder GET + create local + dialog), funcional. El main.dart es byte-identico al de Julian David: evidencia de codigo compartido (penalizacion). 4</t>
+      <c r="C7" s="3">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App de notas Flutter (jsonplaceholder GET + create local + dialog), funcional. El main.dart es byte-identico al de Julian David: evidencia de codigo compartido (penalizacion).</t>
         </is>
       </c>
     </row>
@@ -1195,24 +1290,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAREA 5 - App del Clima (Flutter) 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAREA 5 - App del Clima (Flutter)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rubrica: consumo de OpenWeatherMap, modelo fromJson, manejo de errores, UI y navegacion. Mejor proyecto = 5.0 0</t>
+          <t xml:space="preserve">Rubrica: consumo de OpenWeatherMap, modelo fromJson, manejo de errores, UI y navegacion. Mejor proyecto = 5.0</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle / Justificacion</t>
         </is>
       </c>
     </row>
@@ -1227,12 +1337,12 @@
           <t xml:space="preserve">Marin708/Talleres_Dispositivos_moviles (Evaluacion_1)</t>
         </is>
       </c>
-      <c r="C5">
-        <v>5 3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App del clima (OpenWeatherMap) con ClimaService, manejo de errores 401/404, pantallas Home/Buscar/Detalle. Mejor formato de codigo. Nota: API key hardcodeada (mala practica de seguridad). 4</t>
+      <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App del clima (OpenWeatherMap) con ClimaService, manejo de errores 401/404, pantallas Home/Buscar/Detalle. Mejor formato de codigo. Nota: API key hardcodeada (mala practica de seguridad).</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1357,12 @@
           <t xml:space="preserve">BSM2003/Dispositivos_Moviles (clima)</t>
         </is>
       </c>
-      <c r="C6">
-        <v>4.5 3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App del clima (OpenWeatherMap), modelo Clima.fromJson con emoji por icono, manejo de errores muy completo (404/401/SocketException), 3 pantallas + favoritos. Codigo con indentacion desordenada y API key hardcodeada. 4</t>
+      <c r="C6" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">App del clima (OpenWeatherMap), modelo Clima.fromJson con emoji por icono, manejo de errores muy completo (404/401/SocketException), 3 pantallas + favoritos. Codigo con indentacion desordenada y API key hardcodeada.</t>
         </is>
       </c>
     </row>
@@ -1270,24 +1380,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAREA 6 - Ejercicios de Kotlin / Mi Primera App 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAREA 6 - Ejercicios de Kotlin / Mi Primera App</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rubrica: ejercicios de null safety/Elvis, when, colecciones y data class (parte 3 del taller Kotlin). Mejor proyecto = 5.0 0</t>
+          <t xml:space="preserve">Rubrica: ejercicios de null safety/Elvis, when, colecciones y data class (parte 3 del taller Kotlin). Mejor proyecto = 5.0</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="System.Object[] S" t="inlineStr">
-        <is>
-          <t xml:space="preserve">System.Object[] S</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estudiante</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle / Justificacion</t>
         </is>
       </c>
     </row>
@@ -1302,12 +1427,12 @@
           <t xml:space="preserve">Jumgarciama/MiPrimeraApp</t>
         </is>
       </c>
-      <c r="C5">
-        <v>5 3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Primera App Android con 4 ejercicios de Kotlin correctos: describirEstudiante (Elvis), calcularDescuento (when), filtrado/orden de estudiantes (filter/sortedByDescending/map), resumenCarrito (data class + sumOf). Domina fundamentos. 4</t>
+      <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primera App Android con 4 ejercicios de Kotlin correctos: describirEstudiante (Elvis), calcularDescuento (when), filtrado/orden de estudiantes (filter/sortedByDescending/map), resumenCarrito (data class + sumOf). Domina fundamentos.</t>
         </is>
       </c>
     </row>
@@ -1322,12 +1447,12 @@
           <t xml:space="preserve">JuanCamiloGanan/Programacion-para-dispositivos-moviles (Mi Primera App)</t>
         </is>
       </c>
-      <c r="C6">
-        <v>5 3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ejercicios de fundamentos Kotlin en Ejercicios_1_4.kt: nullable/Elvis, when descuento, filtrado de estudiantes, data class Producto + resumen carrito. Correctos y completos. 4</t>
+      <c r="C6" s="3">
+        <v>5</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ejercicios de fundamentos Kotlin en Ejercicios_1_4.kt: nullable/Elvis, when descuento, filtrado de estudiantes, data class Producto + resumen carrito. Correctos y completos.</t>
         </is>
       </c>
     </row>
@@ -1342,9 +1467,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOTAS Y OBSERVACIONES GENERALES 1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOTAS Y OBSERVACIONES GENERALES</t>
         </is>
       </c>
     </row>
@@ -1352,94 +1477,94 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">- El Parcial 1 (App Tienda con FakeStore API) NO se recalifico aqui: ya fue evaluado por el docente en el archivo original. 0</t>
+          <t xml:space="preserve">- El Parcial 1 (App Tienda con FakeStore API) NO se recalifico aqui: ya fue evaluado por el docente en el archivo original.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">- El Parcial 2 es un cuestionario de seleccion multiple, no genera proyectos en repositorio. 0</t>
+          <t xml:space="preserve">- El Parcial 2 es un cuestionario de seleccion multiple, no genera proyectos en repositorio.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Criterio de calificacion: dentro de cada tarea, el mejor proyecto recibe 5.0 y los demas se escalan segun completitud y calidad. 0</t>
+          <t xml:space="preserve">- Criterio de calificacion: dentro de cada tarea, el mejor proyecto recibe 5.0 y los demas se escalan segun completitud y calidad.</t>
         </is>
       </c>
     </row>
     <row r="6"/>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Casos especiales: 2</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casos especiales:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Vanessa Miranda: el repo de ejercicios (ejercicios-moviles-clase) esta vacio (sin lib/, sin main.dart, sin pubspec). No hay tareas evaluables. 0</t>
+          <t xml:space="preserve">- Vanessa Miranda: el repo de ejercicios (ejercicios-moviles-clase) esta vacio (sin lib/, sin main.dart, sin pubspec). No hay tareas evaluables.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Sofia Calvijo Zuluaga: solo tiene Parcial 1 y una lista-de-tareas en repo aparte no clonado en esta revision; sin tareas adicionales evaluadas aqui. 0</t>
+          <t xml:space="preserve">- Sofia Calvijo Zuluaga: solo tiene Parcial 1 y una lista-de-tareas en repo aparte; sin tareas adicionales evaluadas aqui.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Jeison David Gomez Hernandez: solo entrego App_Tienda (Parcial 1); sin otras tareas en repositorio. 0</t>
+          <t xml:space="preserve">- Jeison David Gomez Hernandez: solo entrego App_Tienda (Parcial 1); sin otras tareas en repositorio.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Jumgarciama/Tareas_flutter: son archivos .zip; uno (ejercicioPrueba.zip) contiene material/ejemplos del profesor, no trabajo propio claro. No evaluado como tarea independiente. 0</t>
+          <t xml:space="preserve">- Jumgarciama/Tareas_flutter: son archivos .zip; uno (ejercicioPrueba.zip) contiene material/ejemplos del profesor, no trabajo propio claro. No evaluado.</t>
         </is>
       </c>
     </row>
     <row r="12"/>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidencias de codigo compartido / copiado (penalizado): 2</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evidencias de codigo compartido / copiado (penalizado):</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Taller Kotlin Lista de Tareas: el de Juan Camilo Ganan es identico al de Veronica Clavijo. 0</t>
+          <t xml:space="preserve">- Taller Kotlin Lista de Tareas: el de Juan Camilo Ganan es identico al de Veronica Clavijo.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">- App de Notas Flutter: el main.dart de Juan Camilo Ganan y el de Julian David son identicos. 0</t>
+          <t xml:space="preserve">- App de Notas Flutter: el main.dart de Juan Camilo Ganan y el de Julian David son identicos.</t>
         </is>
       </c>
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mala practica detectada: 2</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mala practica detectada:</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">- API keys hardcodeadas en las apps del clima de Gustavo Marin y Bryan Salinas (OpenWeatherMap). 0</t>
+          <t xml:space="preserve">- API keys hardcodeadas en las apps del clima de Gustavo Marin y Bryan Salinas (OpenWeatherMap).</t>
         </is>
       </c>
     </row>

</xml_diff>